<commit_message>
[양대용] 사운드 처리작업, 씬 추가(Boot,Title,Stage,Dungeon)
</commit_message>
<xml_diff>
--- a/Shared/XLS/Map.xlsx
+++ b/Shared/XLS/Map.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="6" rupBuild="9303"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="21240"/>
+    <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="21240" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="#Enum" sheetId="6" r:id="rId1"/>
@@ -33,132 +33,132 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="82">
   <si>
     <t>!Enum</t>
-    <phoneticPr fontId="9" type="noConversion"/>
+    <phoneticPr fontId="10" type="noConversion"/>
   </si>
   <si>
     <t>!ID</t>
   </si>
   <si>
     <t xml:space="preserve"> </t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>Name</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>!string</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>!ID</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>!Table</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>MapType</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>Stage</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>Dungeon</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>!int</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>StageNum</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>!int</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>초원</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>!int</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>Desc</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>MapPrefab</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>!string</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>BGM</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>ReqKillCount</t>
   </si>
   <si>
     <t>StageStep</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>Map_1</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>Sound_Map_1</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>EliteMonsterIDs</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>BossMonsterID</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>StepStatMultiplier</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>!float</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>빙하</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>용암</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>빙하지역입니다.</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>초원지역입니다.</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>용암지역입니다.</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>Map_2</t>
@@ -174,35 +174,35 @@
   </si>
   <si>
     <t>101;102;103;104;105</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>106;107;108;109;110</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>111;112;113;114;115</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>DungeonType</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>Gold</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>Exp</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>DungeonType</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>!DungeonType</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <r>
@@ -218,39 +218,39 @@
       </rPr>
       <t>ame</t>
     </r>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>Desc</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>!string</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>Raid</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>TicketItemID</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>TicketCost</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>UnlockCondition</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>DungeonList</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>DungeonStage</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <r>
@@ -266,75 +266,75 @@
       </rPr>
       <t>tep</t>
     </r>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>LimitTime</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>SpawnCount</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>StatMultiplier</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>RewardID</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>!float</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>NormalMonsterIDs</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>DungeonListID</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>골드던전</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>경험치던전</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>레이드</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>Gold</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>Exp</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>Raid</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>경험치를 대량으로 획득 할 수 있는 던전</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>골드를 대량으로 획득 할 수 있는 던전</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>레이드 보스의 데미지를 누적하는 던전</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>퀘스트1제한</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>퀘스트2제한</t>
@@ -344,7 +344,7 @@
   </si>
   <si>
     <t>Dungeon_1</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>Dungeon_2</t>
@@ -354,15 +354,15 @@
   </si>
   <si>
     <t>!Table</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>ClearRewardID</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <t>!int</t>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
   <si>
     <r>
@@ -379,7 +379,27 @@
       </rPr>
       <t>tageInfo</t>
     </r>
-    <phoneticPr fontId="8" type="noConversion"/>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>101;102;103</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>10001</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>;10002</t>
+    </r>
+    <phoneticPr fontId="9" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -389,12 +409,20 @@
   <numFmts count="1">
     <numFmt numFmtId="176" formatCode="mm&quot;월&quot;\ dd&quot;일&quot;"/>
   </numFmts>
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="맑은 고딕"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="맑은 고딕"/>
+      <family val="2"/>
+      <charset val="129"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -576,13 +604,13 @@
   </borders>
   <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -598,43 +626,43 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="3" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="3" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="2" xfId="2" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="2" xfId="2" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="2" xfId="2" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="2" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="5" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="5" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="5" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="5" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -979,7 +1007,7 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="8" type="noConversion"/>
+  <phoneticPr fontId="9" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1231,7 +1259,7 @@
       <c r="E8" s="14"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="8" type="noConversion"/>
+  <phoneticPr fontId="9" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
@@ -1454,7 +1482,7 @@
       <c r="J10" s="5"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="8" type="noConversion"/>
+  <phoneticPr fontId="9" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1610,10 +1638,18 @@
       <c r="E4" s="5">
         <v>120</v>
       </c>
-      <c r="F4" s="5"/>
-      <c r="G4" s="5"/>
-      <c r="H4" s="5"/>
-      <c r="I4" s="5"/>
+      <c r="F4" t="s">
+        <v>80</v>
+      </c>
+      <c r="G4" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="H4" s="5">
+        <v>1000001</v>
+      </c>
+      <c r="I4" s="5">
+        <v>1</v>
+      </c>
       <c r="J4" s="5">
         <v>0.1</v>
       </c>
@@ -1638,6 +1674,18 @@
       <c r="E5" s="5">
         <v>120</v>
       </c>
+      <c r="F5" t="s">
+        <v>80</v>
+      </c>
+      <c r="G5" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="H5" s="5">
+        <v>1000001</v>
+      </c>
+      <c r="I5" s="5">
+        <v>1</v>
+      </c>
       <c r="J5" s="2">
         <v>0.2</v>
       </c>
@@ -1658,6 +1706,18 @@
       <c r="E6" s="5">
         <v>120</v>
       </c>
+      <c r="F6" t="s">
+        <v>80</v>
+      </c>
+      <c r="G6" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="H6" s="5">
+        <v>1000001</v>
+      </c>
+      <c r="I6" s="5">
+        <v>1</v>
+      </c>
       <c r="J6" s="2">
         <v>0.3</v>
       </c>
@@ -1678,6 +1738,18 @@
       <c r="E7" s="5">
         <v>120</v>
       </c>
+      <c r="F7" t="s">
+        <v>80</v>
+      </c>
+      <c r="G7" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="H7" s="5">
+        <v>1000001</v>
+      </c>
+      <c r="I7" s="5">
+        <v>1</v>
+      </c>
       <c r="J7" s="2">
         <v>0.4</v>
       </c>
@@ -1698,6 +1770,18 @@
       <c r="E8" s="5">
         <v>120</v>
       </c>
+      <c r="F8" t="s">
+        <v>80</v>
+      </c>
+      <c r="G8" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="H8" s="5">
+        <v>1000001</v>
+      </c>
+      <c r="I8" s="5">
+        <v>1</v>
+      </c>
       <c r="J8" s="2">
         <v>0.5</v>
       </c>
@@ -1718,6 +1802,18 @@
       <c r="E9" s="5">
         <v>120</v>
       </c>
+      <c r="F9" t="s">
+        <v>80</v>
+      </c>
+      <c r="G9" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="H9" s="5">
+        <v>1000001</v>
+      </c>
+      <c r="I9" s="5">
+        <v>1</v>
+      </c>
       <c r="J9" s="5">
         <v>0.1</v>
       </c>
@@ -1736,6 +1832,18 @@
       <c r="E10" s="5">
         <v>120</v>
       </c>
+      <c r="F10" t="s">
+        <v>80</v>
+      </c>
+      <c r="G10" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="H10" s="5">
+        <v>1000001</v>
+      </c>
+      <c r="I10" s="5">
+        <v>1</v>
+      </c>
       <c r="J10" s="2">
         <v>0.2</v>
       </c>
@@ -1754,6 +1862,18 @@
       <c r="E11" s="5">
         <v>120</v>
       </c>
+      <c r="F11" t="s">
+        <v>80</v>
+      </c>
+      <c r="G11" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="H11" s="5">
+        <v>1000001</v>
+      </c>
+      <c r="I11" s="5">
+        <v>1</v>
+      </c>
       <c r="J11" s="2">
         <v>0.3</v>
       </c>
@@ -1771,6 +1891,18 @@
       <c r="E12" s="5">
         <v>120</v>
       </c>
+      <c r="F12" t="s">
+        <v>80</v>
+      </c>
+      <c r="G12" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="H12" s="5">
+        <v>1000001</v>
+      </c>
+      <c r="I12" s="5">
+        <v>1</v>
+      </c>
       <c r="J12" s="2">
         <v>0.4</v>
       </c>
@@ -1788,6 +1920,18 @@
       <c r="E13" s="5">
         <v>120</v>
       </c>
+      <c r="F13" t="s">
+        <v>80</v>
+      </c>
+      <c r="G13" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="H13" s="5">
+        <v>1000001</v>
+      </c>
+      <c r="I13" s="5">
+        <v>1</v>
+      </c>
       <c r="J13" s="2">
         <v>0.5</v>
       </c>
@@ -1805,6 +1949,18 @@
       <c r="E14" s="5">
         <v>120</v>
       </c>
+      <c r="F14" t="s">
+        <v>80</v>
+      </c>
+      <c r="G14" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="H14" s="5">
+        <v>1000001</v>
+      </c>
+      <c r="I14" s="5">
+        <v>1</v>
+      </c>
       <c r="J14" s="5">
         <v>0.1</v>
       </c>
@@ -1822,6 +1978,18 @@
       <c r="E15" s="5">
         <v>120</v>
       </c>
+      <c r="F15" t="s">
+        <v>80</v>
+      </c>
+      <c r="G15" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="H15" s="5">
+        <v>1000001</v>
+      </c>
+      <c r="I15" s="5">
+        <v>1</v>
+      </c>
       <c r="J15" s="2">
         <v>0.2</v>
       </c>
@@ -1839,6 +2007,18 @@
       <c r="E16" s="5">
         <v>120</v>
       </c>
+      <c r="F16" t="s">
+        <v>80</v>
+      </c>
+      <c r="G16" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="H16" s="5">
+        <v>1000001</v>
+      </c>
+      <c r="I16" s="5">
+        <v>1</v>
+      </c>
       <c r="J16" s="2">
         <v>0.3</v>
       </c>
@@ -1856,6 +2036,18 @@
       <c r="E17" s="5">
         <v>120</v>
       </c>
+      <c r="F17" t="s">
+        <v>80</v>
+      </c>
+      <c r="G17" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="H17" s="5">
+        <v>1000001</v>
+      </c>
+      <c r="I17" s="5">
+        <v>1</v>
+      </c>
       <c r="J17" s="2">
         <v>0.4</v>
       </c>
@@ -1873,12 +2065,24 @@
       <c r="E18" s="5">
         <v>120</v>
       </c>
+      <c r="F18" t="s">
+        <v>80</v>
+      </c>
+      <c r="G18" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="H18" s="5">
+        <v>1000001</v>
+      </c>
+      <c r="I18" s="5">
+        <v>1</v>
+      </c>
       <c r="J18" s="2">
         <v>0.5</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="8" type="noConversion"/>
+  <phoneticPr fontId="9" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>